<commit_message>
Auto update claims data - Thu 08/06/2026 22:00:02.36
</commit_message>
<xml_diff>
--- a/ميدسيرفس.xlsx
+++ b/ميدسيرفس.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Pharmacy_Operations\Insurance_Accounts\Insurance_Claims\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77164BA9-E866-4FC6-863F-75B6E1AD4A1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{470A3930-43C1-4966-98CA-0B415DF149B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D788D8F7-2544-4C2F-9B89-70931910278C}"/>
   </bookViews>
@@ -751,21 +751,6 @@
   </cellStyles>
   <dxfs count="27">
     <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.000\ _د_._ا_._‏_-;\-* #,##0.000\ _د_._ا_._‏_-;_-* &quot;-&quot;???\ _د_._ا_._‏_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.000\ _د_._ا_._‏_-;\-* #,##0.000\ _د_._ا_._‏_-;_-* &quot;-&quot;???\ _د_._ا_._‏_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.000\ _د_._ا_._‏_-;\-* #,##0.000\ _د_._ا_._‏_-;_-* &quot;-&quot;???\ _د_._ا_._‏_-;_-@_-"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="164" formatCode="_-* #,##0.000\ _د_._ا_._‏_-;\-* #,##0.000\ _د_._ا_._‏_-;_-* &quot;-&quot;???\ _د_._ا_._‏_-;_-@_-"/>
     </dxf>
     <dxf>
@@ -810,6 +795,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.000\ _د_._ا_._‏_-;\-* #,##0.000\ _د_._ا_._‏_-;_-* &quot;-&quot;???\ _د_._ا_._‏_-;_-@_-"/>
     </dxf>
     <dxf>
       <font>
@@ -828,6 +814,21 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.000\ _د_._ا_._‏_-;\-* #,##0.000\ _د_._ا_._‏_-;_-* &quot;-&quot;???\ _د_._ا_._‏_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.000\ _د_._ا_._‏_-;\-* #,##0.000\ _د_._ا_._‏_-;_-* &quot;-&quot;???\ _د_._ا_._‏_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.000\ _د_._ا_._‏_-;\-* #,##0.000\ _د_._ا_._‏_-;_-* &quot;-&quot;???\ _د_._ا_._‏_-;_-@_-"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="_-* #,##0.000\ _د_._ا_._‏_-;\-* #,##0.000\ _د_._ا_._‏_-;_-* &quot;-&quot;???\ _د_._ا_._‏_-;_-@_-"/>
     </dxf>
     <dxf>
@@ -865,7 +866,6 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.000\ _د_._ا_._‏_-;\-* #,##0.000\ _د_._ا_._‏_-;_-* &quot;-&quot;???\ _د_._ا_._‏_-;_-@_-"/>
     </dxf>
     <dxf>
       <font>
@@ -1154,19 +1154,19 @@
     <tableColumn id="4" xr3:uid="{4FA0F61B-0974-4290-8AF9-64F3425CF95F}" name="رقم النموذج" dataDxfId="19" totalsRowDxfId="18"/>
     <tableColumn id="5" xr3:uid="{FA7C7B11-59CD-43FE-8614-AE77C814F7B1}" name="نوع المستفيد" dataDxfId="17" totalsRowDxfId="16"/>
     <tableColumn id="6" xr3:uid="{A5C7FB1D-369A-430A-90FD-DECEB437BB07}" name="تاريخ البيع" dataDxfId="15" totalsRowDxfId="14"/>
-    <tableColumn id="7" xr3:uid="{A0C6C549-4E6F-40C8-8B90-0D7D85B722AF}" name="قيمة الفاتورة" dataDxfId="13" totalsRowDxfId="12"/>
-    <tableColumn id="8" xr3:uid="{FE5B0B26-736F-4D13-A599-E33B398493F1}" name="قيمة المشاركة" dataDxfId="11" totalsRowDxfId="10"/>
-    <tableColumn id="9" xr3:uid="{BC1FF825-92ED-4149-A1D2-B9B13F698346}" name="صافي القيمة" dataDxfId="9" totalsRowDxfId="8"/>
-    <tableColumn id="10" xr3:uid="{856C6145-2E1C-4B6E-9442-8F25AAAF88C3}" name="القيمة المطلوبة" totalsRowFunction="sum" dataDxfId="7" totalsRowDxfId="6">
+    <tableColumn id="7" xr3:uid="{A0C6C549-4E6F-40C8-8B90-0D7D85B722AF}" name="قيمة الفاتورة" dataDxfId="13" totalsRowDxfId="5"/>
+    <tableColumn id="8" xr3:uid="{FE5B0B26-736F-4D13-A599-E33B398493F1}" name="قيمة المشاركة" dataDxfId="12" totalsRowDxfId="4"/>
+    <tableColumn id="9" xr3:uid="{BC1FF825-92ED-4149-A1D2-B9B13F698346}" name="صافي القيمة" dataDxfId="11" totalsRowDxfId="3"/>
+    <tableColumn id="10" xr3:uid="{856C6145-2E1C-4B6E-9442-8F25AAAF88C3}" name="القيمة المطلوبة" totalsRowFunction="sum" dataDxfId="10" totalsRowDxfId="2">
       <calculatedColumnFormula>G2*0.94-H2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{93671F58-AEBB-42C2-8ECB-4A20CA480AFD}" name="المدفوع" totalsRowFunction="sum" dataDxfId="5" totalsRowDxfId="4">
+    <tableColumn id="11" xr3:uid="{93671F58-AEBB-42C2-8ECB-4A20CA480AFD}" name="المدفوع" totalsRowFunction="sum" dataDxfId="9" totalsRowDxfId="1">
       <calculatedColumnFormula>Table1[[#This Row],[القيمة المطلوبة]]*0.9557</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{3CB96BCB-F76A-4AB9-8336-BDA8FF662F9F}" name="المتبقي" dataDxfId="3" totalsRowDxfId="2">
+    <tableColumn id="12" xr3:uid="{3CB96BCB-F76A-4AB9-8336-BDA8FF662F9F}" name="المتبقي" dataDxfId="8" totalsRowDxfId="0">
       <calculatedColumnFormula>J2-K2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{5DF86495-E104-4E7E-9037-241357A5F93D}" name="تاريخ الدفعة" dataDxfId="1" totalsRowDxfId="0"/>
+    <tableColumn id="13" xr3:uid="{5DF86495-E104-4E7E-9037-241357A5F93D}" name="تاريخ الدفعة" dataDxfId="7" totalsRowDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -7516,7 +7516,7 @@
         <v>13.807953599999999</v>
       </c>
       <c r="L162" s="6">
-        <f t="shared" ref="L162:L193" si="12">J162-K162</f>
+        <f t="shared" ref="L162:L180" si="12">J162-K162</f>
         <v>0.64004639999999924</v>
       </c>
       <c r="M162" s="7">
@@ -7916,7 +7916,7 @@
         <v>1.5678212999999985</v>
       </c>
       <c r="M171" s="7">
-        <v>46240</v>
+        <v>46239</v>
       </c>
     </row>
     <row r="172" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
@@ -7960,7 +7960,7 @@
         <v>0.13965132000000002</v>
       </c>
       <c r="M172" s="7">
-        <v>46240</v>
+        <v>46239</v>
       </c>
     </row>
     <row r="173" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
@@ -8004,7 +8004,7 @@
         <v>0.26323946000000031</v>
       </c>
       <c r="M173" s="7">
-        <v>46240</v>
+        <v>46239</v>
       </c>
     </row>
     <row r="174" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">
@@ -8048,7 +8048,7 @@
         <v>1.6812381599999995</v>
       </c>
       <c r="M174" s="7">
-        <v>46240</v>
+        <v>46239</v>
       </c>
     </row>
     <row r="175" spans="1:13" ht="14.4" x14ac:dyDescent="0.3">

</xml_diff>